<commit_message>
Actualizacao das paginas de feiras
</commit_message>
<xml_diff>
--- a/Beneficiarios_Indiretos.xlsx
+++ b/Beneficiarios_Indiretos.xlsx
@@ -1519,13 +1519,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C435ABF6-8F8B-432C-B87D-A465B9D10D97}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1B9D8538-371B-471E-8E88-256500138BA7}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18F3E3D0-74D6-4AF9-B583-827E2345B594}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECE78F7C-D429-491C-8238-C328925DA51E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{553813F4-364F-4482-8625-B138E47CA708}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC8F0C7E-7CBF-429F-83C7-D6AFFEFDD276}"/>
 </file>
</xml_diff>